<commit_message>
feat(pmer): update permission in queries
</commit_message>
<xml_diff>
--- a/static/files/create-team-member-template.xlsx
+++ b/static/files/create-team-member-template.xlsx
@@ -11447,17 +11447,13 @@
       <c r="I1001" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ede9"/>
-  <dataValidations count="3">
-    <dataValidation allowBlank="true" error="Please select MALE or FEMALE from the dropdown." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D3:D1001" type="list">
-      <formula1>"MALE,FEMALE"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
+  <sheetProtection sheet="true" password="ede9" objects="true" scenarios="true"/>
+  <dataValidations count="2">
     <dataValidation allowBlank="true" error="Please select a region from the dropdown. New regions must be added on the Lists sheet by the administrator." errorStyle="stop" errorTitle="Invalid region" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F1001" type="list">
       <formula1>Regions</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please select MALE or FEMALE from the dropdown." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2" type="list">
+    <dataValidation allowBlank="true" error="Please select MALE or FEMALE from the dropdown." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D1:D1001" type="list">
       <formula1>"MALE,FEMALE,OTHER"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11481,6 +11477,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11554,7 +11551,13 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ede9"/>
+  <sheetProtection sheet="true" password="ede9" objects="true" scenarios="true"/>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" error="Please select MALE or FEMALE from the dropdown." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C1:C1014" type="list">
+      <formula1>$b1$b3</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>